<commit_message>
Bugs fixed post testing on exp. DM2
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -1,25 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748D77CF-59EF-4F18-A53E-022E7480E160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="139">
   <si>
     <t>Section</t>
   </si>
@@ -61,9 +67,6 @@
   </si>
   <si>
     <t>Input folder:</t>
-  </si>
-  <si>
-    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/ORG slices contr females 13.4.26/Analysis/</t>
   </si>
   <si>
     <t>Folder path as text. 
@@ -114,9 +117,6 @@
     <t>Sample names:</t>
   </si>
   <si>
-    <t>["Liver1", "Liver2", "Kid1", "Kid2", "Lung1", "Lung2"]</t>
-  </si>
-  <si>
     <t>List of group names, or None. 
 Example: ["Liver1", "Liver2"]</t>
   </si>
@@ -130,9 +130,6 @@
     <t>Include all files:</t>
   </si>
   <si>
-    <t>False</t>
-  </si>
-  <si>
     <t>True / False</t>
   </si>
   <si>
@@ -161,9 +158,6 @@
     <t>Remove background noise:</t>
   </si>
   <si>
-    <t>True</t>
-  </si>
-  <si>
     <t>True = subtract the average pre-sample noise from the signal. False = keep the signal without subtracting that background.</t>
   </si>
   <si>
@@ -275,9 +269,6 @@
     <t>Choose plot style:</t>
   </si>
   <si>
-    <t>line</t>
-  </si>
-  <si>
     <t>points / line / points+line</t>
   </si>
   <si>
@@ -306,9 +297,6 @@
     <t>Plot description:</t>
   </si>
   <si>
-    <t>Control (females 13.4.26)</t>
-  </si>
-  <si>
     <t>Text, or None.</t>
   </si>
   <si>
@@ -472,17 +460,29 @@
   </si>
   <si>
     <t>override_visible_replicate_cols</t>
+  </si>
+  <si>
+    <t>["10% serum", "2% serum", "20% serum", "Dex - 10% serum", "Allicin 1", "Allicin 10", "Allicin 25", "Allicin 10 (26.3)", "Allicin 25 (26.3)"]</t>
+  </si>
+  <si>
+    <t>points</t>
+  </si>
+  <si>
+    <t>DM2</t>
+  </si>
+  <si>
+    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/DM2/Analysis/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -490,7 +490,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -498,7 +498,7 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -506,14 +506,14 @@
       <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -521,7 +521,7 @@
       <b/>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -591,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -602,9 +602,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -623,19 +620,33 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -673,7 +684,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -707,6 +718,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -741,9 +753,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -916,17 +929,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="4" width="42.7109375" customWidth="1"/>
-    <col min="5" max="5" width="75.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.69921875" customWidth="1"/>
+    <col min="2" max="4" width="42.69921875" customWidth="1"/>
+    <col min="5" max="5" width="75.69921875" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -946,706 +959,685 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="20" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="5" t="s">
+    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="20" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="20" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="8">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="9">
-        <v>5</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="6" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="96" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="F8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="6" t="s">
+    </row>
+    <row r="9" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="C9" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="8" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="C11" s="8">
+        <v>20</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="9">
-        <v>25</v>
-      </c>
-      <c r="D11" s="8" t="s">
+    </row>
+    <row r="12" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="C12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
+    <row r="13" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="20" customHeight="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="F14" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="7" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6" t="s">
+      <c r="F15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="7" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="E16" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="7" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="B18" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="C18" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F18" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
+    <row r="19" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="C20" s="8">
+        <v>10</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="E20" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="6" t="s">
+    </row>
+    <row r="21" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="9">
-        <v>10</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C21" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F21" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
+    <row r="22" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C21" s="9">
-        <v>7</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="B23" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="C23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F23" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="5" t="s">
+    <row r="24" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C24" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="6" t="s">
+      <c r="E24" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F24" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
+    <row r="25" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E25" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F25" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
+    <row r="26" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C26" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="E26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F26" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F25" s="6" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="5" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
+      <c r="C27" s="8">
+        <v>0</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="E27" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="F27" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E26" s="6" t="s">
+    </row>
+    <row r="28" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="C28" s="8">
+        <v>0</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6" t="s">
+      <c r="E28" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C27" s="9">
-        <v>6</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="F28" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E27" s="6" t="s">
+    </row>
+    <row r="29" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+    </row>
+    <row r="30" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+      <c r="C30" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="9">
+      <c r="F30" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
+      <c r="B31" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="F28" s="6" t="s">
+      <c r="D31" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="20" customHeight="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="5" t="s">
+      <c r="F31" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B30" s="6" t="s">
+    </row>
+    <row r="32" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" s="6" t="s">
+      <c r="C32" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F32" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="5"/>
-      <c r="B31" s="6" t="s">
+    <row r="33" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+    </row>
+    <row r="34" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="C31" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E31" s="6" t="s">
+      <c r="B34" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="C34" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E34" s="5" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6" t="s">
+      <c r="F34" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E32" s="6" t="s">
+    </row>
+    <row r="35" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="C35" s="8">
+        <v>2</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="20" customHeight="1">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="F35" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" s="6" t="s">
+    </row>
+    <row r="36" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+    </row>
+    <row r="37" spans="1:6" ht="204.6" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="B37" s="5" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="5"/>
-      <c r="B35" s="6" t="s">
+      <c r="C37" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C35" s="9">
-        <v>2</v>
-      </c>
-      <c r="D35" s="8" t="s">
+      <c r="D37" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E37" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F37" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="20" customHeight="1">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="5" t="s">
+    <row r="38" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A38" s="10"/>
+      <c r="B38" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="C38" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D38" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="E38" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="F38" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="E37" s="6" t="s">
+    </row>
+    <row r="39" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A39" s="10"/>
+      <c r="B39" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="E39" s="5" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="5"/>
-      <c r="B38" s="6" t="s">
+      <c r="F39" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C38" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="8" t="s">
+    </row>
+    <row r="40" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="C40" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="E40" s="5" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5"/>
-      <c r="B39" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D39" s="8" t="s">
+      <c r="F40" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="6" t="s">
+    </row>
+    <row r="41" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="F39" s="6" t="s">
+      <c r="C41" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="5"/>
-      <c r="B40" s="6" t="s">
+      <c r="E41" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D40" s="8" t="s">
+      <c r="F41" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="E40" s="6" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="C42" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="5"/>
-      <c r="B41" s="6" t="s">
+      <c r="E42" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D41" s="8" t="s">
+      <c r="F42" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="5"/>
-      <c r="B42" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="19">
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A37:A42"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:A42"/>
   </mergeCells>
-  <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C34 C30:C32 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C12">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C18">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C23">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"points,line,points+line"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C30">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C32">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C34">
-      <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added display settings to allow showing the average without replicates
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748D77CF-59EF-4F18-A53E-022E7480E160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E18A45-D828-4AA6-8262-3AF96710CC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="146">
   <si>
     <t>Section</t>
   </si>
@@ -130,6 +130,9 @@
     <t>Include all files:</t>
   </si>
   <si>
+    <t>False</t>
+  </si>
+  <si>
     <t>True / False</t>
   </si>
   <si>
@@ -158,6 +161,9 @@
     <t>Remove background noise:</t>
   </si>
   <si>
+    <t>True</t>
+  </si>
+  <si>
     <t>True = subtract the average pre-sample noise from the signal. False = keep the signal without subtracting that background.</t>
   </si>
   <si>
@@ -266,6 +272,18 @@
     <t>plot_raw_data</t>
   </si>
   <si>
+    <t>Replicate display mode:</t>
+  </si>
+  <si>
+    <t>replicates_and_mean / mean_only / replicates_only</t>
+  </si>
+  <si>
+    <t>Choose what to display on the raw-data plots. replicates_and_mean = show both replicates and the average signal. mean_only = show only the average signal. replicates_only = show only the replicate signals, without the average.</t>
+  </si>
+  <si>
+    <t>replicate_display_mode</t>
+  </si>
+  <si>
     <t>Choose plot style:</t>
   </si>
   <si>
@@ -462,16 +480,19 @@
     <t>override_visible_replicate_cols</t>
   </si>
   <si>
+    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/DM2/Analysis/</t>
+  </si>
+  <si>
     <t>["10% serum", "2% serum", "20% serum", "Dex - 10% serum", "Allicin 1", "Allicin 10", "Allicin 25", "Allicin 10 (26.3)", "Allicin 25 (26.3)"]</t>
   </si>
   <si>
-    <t>points</t>
-  </si>
-  <si>
-    <t>DM2</t>
-  </si>
-  <si>
-    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/DM2/Analysis/</t>
+    <t>points+line</t>
+  </si>
+  <si>
+    <t>"DM2"</t>
+  </si>
+  <si>
+    <t>mean_only</t>
   </si>
 </sst>
 </file>
@@ -930,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.69921875" customWidth="1"/>
@@ -975,7 +996,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>8</v>
@@ -1049,7 +1070,7 @@
         <v>22</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>23</v>
@@ -1066,17 +1087,17 @@
       <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="6" t="b">
-        <v>0</v>
+      <c r="C9" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1089,40 +1110,40 @@
     </row>
     <row r="11" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" s="8">
         <v>20</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="6" t="b">
-        <v>1</v>
+        <v>36</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1135,58 +1156,58 @@
     </row>
     <row r="14" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1199,22 +1220,22 @@
     </row>
     <row r="18" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="6" t="b">
-        <v>1</v>
+        <v>57</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1227,40 +1248,40 @@
     </row>
     <row r="20" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C20" s="8">
         <v>10</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1273,354 +1294,372 @@
     </row>
     <row r="23" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" s="6" t="b">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="93" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>76</v>
+        <v>143</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" s="8">
-        <v>0</v>
+        <v>86</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>144</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C28" s="8">
         <v>0</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-    </row>
-    <row r="30" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C30" s="6" t="b">
+    </row>
+    <row r="29" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="8">
         <v>0</v>
       </c>
-      <c r="D30" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="F30" s="5" t="s">
+      <c r="D29" s="7" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
+      <c r="E29" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" ht="37.200000000000003" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>98</v>
+      </c>
       <c r="B31" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C31" s="6" t="b">
         <v>0</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C32" s="6" t="b">
         <v>0</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-    </row>
-    <row r="34" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C34" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E34" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F34" s="5" t="s">
+    </row>
+    <row r="33" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="5" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A35" s="10"/>
+      <c r="C33" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="35" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>108</v>
+      </c>
       <c r="B35" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C35" s="8">
+        <v>109</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A36" s="10"/>
+      <c r="B36" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C36" s="8">
         <v>2</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-    </row>
-    <row r="37" spans="1:6" ht="204.6" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="D37" s="7" t="s">
+      <c r="D36" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F36" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
-      <c r="A38" s="10"/>
+    <row r="37" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" ht="204.6" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
+        <v>116</v>
+      </c>
       <c r="B38" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="55.8" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="5" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="5" t="s">
-        <v>123</v>
+        <v>86</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="93" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
       <c r="B42" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="19">
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:A42"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:A43"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:A33"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:A16"/>
@@ -1632,11 +1671,14 @@
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A10:F10"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C34 C30:C32 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C35 C31:C33 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24" xr:uid="{00000000-0002-0000-0000-000004000000}">
+      <formula1>"replicates_and_mean,mean_only,replicates_only"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"points,line,points+line"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Several bug fixes with plotting
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -1,25 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46299D3B-DA6B-4567-9774-E8ED6FE8EB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="8340" yWindow="108" windowWidth="14700" windowHeight="12132" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="144">
   <si>
     <t>Section</t>
   </si>
@@ -65,7 +71,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -75,7 +81,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -105,7 +111,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -115,7 +121,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -123,9 +129,6 @@
     </r>
   </si>
   <si>
-    <t>analysis_output</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 Folder name 
 or 
@@ -149,7 +152,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -159,7 +162,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -689,16 +692,28 @@
   <si>
     <t>override_visible_replicate_cols</t>
   </si>
+  <si>
+    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/DM3/Analysis/</t>
+  </si>
+  <si>
+    <t>DM3 Analysis</t>
+  </si>
+  <si>
+    <t>["25", "c", "dex 25", "dex"]</t>
+  </si>
+  <si>
+    <t>"DM3 Analysis"</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -706,7 +721,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -714,7 +729,7 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -722,14 +737,14 @@
       <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -737,7 +752,7 @@
       <b/>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -746,6 +761,14 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -807,7 +830,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -818,9 +841,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -839,19 +859,33 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -889,7 +923,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -923,6 +957,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -957,9 +992,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1132,17 +1168,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="4" width="42.7109375" customWidth="1"/>
-    <col min="5" max="5" width="78.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.69921875" customWidth="1"/>
+    <col min="2" max="4" width="42.69921875" customWidth="1"/>
+    <col min="5" max="5" width="78.69921875" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1162,717 +1198,706 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="20" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="5" t="s">
+    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="20" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="5" t="s">
+    <row r="4" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="20" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="8">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="9">
-        <v>3</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="6" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="6" t="s">
+    </row>
+    <row r="9" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="6" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="8">
+        <v>25</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="9">
-        <v>25</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="6" t="s">
+    </row>
+    <row r="12" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="6" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="20" customHeight="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="6" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="E15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="6" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="E16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F16" s="6" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="6" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="8">
+        <v>10</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="9">
-        <v>10</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="E20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F20" s="6" t="s">
+    </row>
+    <row r="21" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6">
+        <v>7</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="6" t="s">
+    </row>
+    <row r="22" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="5" t="s">
+      <c r="B23" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="6" t="s">
+    </row>
+    <row r="24" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="E24" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="6" t="s">
+    </row>
+    <row r="25" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="5" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="E25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F25" s="6" t="s">
+    </row>
+    <row r="26" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
+      <c r="C26" s="6">
+        <v>8500</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F26" s="6" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="5" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="8" t="s">
+      <c r="E27" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F27" s="6" t="s">
+    </row>
+    <row r="28" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="5" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="8">
+        <v>0</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="9">
+      <c r="E28" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="8">
         <v>0</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="5"/>
-      <c r="B29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="9">
-        <v>0</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="E29" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="F29" s="6" t="s">
+    </row>
+    <row r="30" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="F31" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="F32" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="5"/>
-      <c r="B33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="F33" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="35" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D33" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="F35" s="6" t="s">
+    </row>
+    <row r="36" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A36" s="10"/>
+      <c r="B36" s="5" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="5"/>
-      <c r="B36" s="6" t="s">
+      <c r="C36" s="8">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="9">
-        <v>2</v>
-      </c>
-      <c r="D36" s="8" t="s">
+      <c r="E36" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F36" s="6" t="s">
+    </row>
+    <row r="37" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" ht="316.2" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="20" customHeight="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="5" t="s">
+      <c r="B38" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="C38" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="D38" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="E38" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F38" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="F38" s="6" t="s">
+    </row>
+    <row r="39" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A39" s="10"/>
+      <c r="B39" s="5" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5"/>
-      <c r="B39" s="6" t="s">
+      <c r="C39" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C39" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39" s="8" t="s">
+      <c r="E39" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="F39" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="F39" s="6" t="s">
+    </row>
+    <row r="40" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="5"/>
-      <c r="B40" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D40" s="8" t="s">
+      <c r="E40" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="F40" s="6" t="s">
+    </row>
+    <row r="41" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="5" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="5"/>
-      <c r="B41" s="6" t="s">
+      <c r="C41" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D41" s="8" t="s">
+      <c r="E41" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="F41" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="F41" s="6" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="5" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="5"/>
-      <c r="B42" s="6" t="s">
+      <c r="C42" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D42" s="8" t="s">
+      <c r="E42" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="F42" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F42" s="6" t="s">
+    </row>
+    <row r="43" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="5" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="5"/>
-      <c r="B43" s="6" t="s">
+      <c r="C43" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E43" s="6" t="s">
+      <c r="F43" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="19">
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:A29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:A43"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C35 C31:C33 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C12">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C18">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C23">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"replicates_and_mean,mean_only,replicates_only"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"points,line,points+line"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C32">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C35">
-      <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ready to run from terminal + user guide added
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46299D3B-DA6B-4567-9774-E8ED6FE8EB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBAEB9F-C59D-4E09-9FD0-33E0A9A017A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="108" windowWidth="14700" windowHeight="12132" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-Paste the path to the folder that contains the Lumi raw CSV files. The folder should contain files such as 1a_Raw.csv, 1b_Raw.csv, 2a_Raw.csv, etc.Make sure the backslashes / are in the same direction as here.
+Paste the path to the folder that contains the Lumi raw CSV files. The folder should contain files such as 1a_Raw.csv, 1b_Raw.csv, 2a_Raw.csv, etc.
 </t>
   </si>
   <si>
@@ -1206,7 +1206,7 @@
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
     </row>
-    <row r="3" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="93" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1262,7 +1262,7 @@
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>16</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>64</v>
       </c>
       <c r="C21" s="6">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
Reset the settings file
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -1,31 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBAEB9F-C59D-4E09-9FD0-33E0A9A017A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -43,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="141">
   <si>
     <t>Section</t>
   </si>
@@ -71,7 +65,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -81,7 +75,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -111,7 +105,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -121,7 +115,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -129,6 +123,9 @@
     </r>
   </si>
   <si>
+    <t>analysis_output</t>
+  </si>
+  <si>
     <t xml:space="preserve">
 Folder name 
 or 
@@ -152,7 +149,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -162,7 +159,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Arial"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -692,28 +689,16 @@
   <si>
     <t>override_visible_replicate_cols</t>
   </si>
-  <si>
-    <t>C:/Users/yuval/OneDrive/Desktop/Lumi/DM3/Analysis/</t>
-  </si>
-  <si>
-    <t>DM3 Analysis</t>
-  </si>
-  <si>
-    <t>["25", "c", "dex 25", "dex"]</t>
-  </si>
-  <si>
-    <t>"DM3 Analysis"</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -721,7 +706,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -729,7 +714,7 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -737,14 +722,14 @@
       <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -752,7 +737,7 @@
       <b/>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -761,14 +746,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -830,7 +807,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -841,6 +818,9 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -859,33 +839,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -923,7 +889,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -957,7 +923,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -992,10 +957,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1168,17 +1132,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.69921875" customWidth="1"/>
-    <col min="2" max="4" width="42.69921875" customWidth="1"/>
-    <col min="5" max="5" width="78.69921875" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="78.7109375" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1198,706 +1162,717 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-    </row>
-    <row r="3" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="2" spans="1:6" ht="20" customHeight="1">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7"/>
+      <c r="D3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="20" customHeight="1">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20" customHeight="1">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="9">
+        <v>3</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="20" customHeight="1">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="9">
+        <v>25</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="20" customHeight="1">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="20" customHeight="1">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="20" customHeight="1">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="9">
+        <v>10</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="20" customHeight="1">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="5"/>
+      <c r="B26" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="7"/>
+      <c r="D26" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="5"/>
+      <c r="B27" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="9">
+        <v>0</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29" s="9">
+        <v>0</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="20" customHeight="1">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="5"/>
+      <c r="B32" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="5"/>
+      <c r="B33" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="20" customHeight="1">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="5"/>
+      <c r="B36" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" s="9">
+        <v>2</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="20" customHeight="1">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="5"/>
+      <c r="B39" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="5"/>
+      <c r="B40" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="5"/>
+      <c r="B41" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="5"/>
+      <c r="B42" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="5"/>
+      <c r="B43" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="F43" s="6" t="s">
         <v>140</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-    </row>
-    <row r="5" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-    </row>
-    <row r="7" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="8">
-        <v>3</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
-      <c r="B8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="8">
-        <v>25</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-    </row>
-    <row r="14" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
-      <c r="B15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-    </row>
-    <row r="18" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="8">
-        <v>10</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="10"/>
-      <c r="B21" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="6">
-        <v>9</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-    </row>
-    <row r="23" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
-      <c r="A24" s="10"/>
-      <c r="B24" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A25" s="10"/>
-      <c r="B25" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A26" s="10"/>
-      <c r="B26" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C26" s="6">
-        <v>8500</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A27" s="10"/>
-      <c r="B27" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A28" s="10"/>
-      <c r="B28" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C28" s="8">
-        <v>0</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A29" s="10"/>
-      <c r="B29" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C29" s="8">
-        <v>0</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-    </row>
-    <row r="31" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
-      <c r="B32" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9"/>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-    </row>
-    <row r="35" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="93" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C36" s="8">
-        <v>2</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-    </row>
-    <row r="38" spans="1:6" ht="316.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
-      <c r="A39" s="10"/>
-      <c r="B39" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
-      <c r="A40" s="10"/>
-      <c r="B40" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
-      <c r="B41" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
-      <c r="A42" s="10"/>
-      <c r="B42" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
-      <c r="A43" s="10"/>
-      <c r="B43" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="E43" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="19">
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:A43"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C35 C31:C33 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="10">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C12">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C18">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C23">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
       <formula1>"replicates_and_mean,mean_only,replicates_only"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25">
       <formula1>"points,line,points+line"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C32">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C35">
+      <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Several bug fixes in plotting override functions
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -1,25 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yuval\PycharmProjects\Lumi Analysis\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{466F94C8-7F56-413A-8ABB-D987D060B59A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="1152" yWindow="108" windowWidth="14700" windowHeight="12132" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="147">
   <si>
     <t>Section</t>
   </si>
@@ -65,7 +71,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -75,7 +81,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -105,7 +111,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -115,7 +121,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -123,9 +129,6 @@
     </r>
   </si>
   <si>
-    <t>analysis_output</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 Folder name 
 or 
@@ -149,7 +152,7 @@
         <b/>
         <sz val="20"/>
         <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -159,7 +162,7 @@
       <rPr>
         <sz val="15"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -689,16 +692,37 @@
   <si>
     <t>override_visible_replicate_cols</t>
   </si>
+  <si>
+    <t>C:\Users\yuval\OneDrive\Desktop\Lumi\ORG slices contr females 13.4.26\Analysis</t>
+  </si>
+  <si>
+    <t>["Liver1", "Liver2", "Kid1", "Kid2", "Lung1", "Lung2"]</t>
+  </si>
+  <si>
+    <t>Control (F) 13.04.2026</t>
+  </si>
+  <si>
+    <t>["Kid1", "Kid2", "Liver1", "Liver2", "Lung1", "Lung2"]</t>
+  </si>
+  <si>
+    <t>[250, 250, 200, 200, 400, 600]</t>
+  </si>
+  <si>
+    <t>Control (F) - Override Test</t>
+  </si>
+  <si>
+    <t>[None ,None , ["2a"], ["2c"], None, ["7c"]]</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -706,7 +730,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -714,7 +738,7 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -722,14 +746,14 @@
       <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -737,7 +761,7 @@
       <b/>
       <sz val="15"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -746,6 +770,14 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -807,7 +839,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -818,9 +850,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -839,19 +868,33 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -889,7 +932,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -923,6 +966,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -957,9 +1001,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1132,17 +1177,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="4" width="42.7109375" customWidth="1"/>
-    <col min="5" max="5" width="78.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.69921875" customWidth="1"/>
+    <col min="2" max="4" width="42.69921875" customWidth="1"/>
+    <col min="5" max="5" width="78.69921875" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1162,717 +1207,702 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="20" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="5" t="s">
+    <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="20" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="5" t="s">
+    <row r="4" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="20" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="8">
+        <v>5</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="9">
-        <v>3</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="6" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="6" t="s">
+    </row>
+    <row r="9" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="6" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="8">
+        <v>25</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="9">
-        <v>25</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="6" t="s">
+    </row>
+    <row r="12" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="6" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="20" customHeight="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="6" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="E15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="6" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="E16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F16" s="6" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="6" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="8">
+        <v>10</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="9">
-        <v>10</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="E20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="F20" s="6" t="s">
+    </row>
+    <row r="21" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="5" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6"/>
+      <c r="D21" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="6" t="s">
+    </row>
+    <row r="22" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="5" t="s">
+      <c r="B23" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="6" t="s">
+    </row>
+    <row r="24" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="E24" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="6" t="s">
+    </row>
+    <row r="25" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="5" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="E25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="F25" s="6" t="s">
+    </row>
+    <row r="26" spans="1:6" ht="130.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
+      <c r="C26" s="6"/>
+      <c r="D26" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F26" s="6" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="5" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="8" t="s">
+      <c r="E27" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F27" s="6" t="s">
+    </row>
+    <row r="28" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="5" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="8">
+        <v>6</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="9">
+      <c r="E28" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="8">
         <v>0</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="5"/>
-      <c r="B29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="9">
-        <v>0</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="E29" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="F29" s="6" t="s">
+    </row>
+    <row r="30" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="F31" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="F32" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="5"/>
-      <c r="B33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="F33" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="35" spans="1:6" ht="74.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D33" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="F35" s="6" t="s">
+    </row>
+    <row r="36" spans="1:6" ht="93" x14ac:dyDescent="0.25">
+      <c r="A36" s="10"/>
+      <c r="B36" s="5" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="5"/>
-      <c r="B36" s="6" t="s">
+      <c r="C36" s="8">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="9">
-        <v>2</v>
-      </c>
-      <c r="D36" s="8" t="s">
+      <c r="E36" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F36" s="6" t="s">
+    </row>
+    <row r="37" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" spans="1:6" ht="316.2" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="20" customHeight="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="5" t="s">
+      <c r="B38" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="C38" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A39" s="10"/>
+      <c r="B39" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C38" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="F38" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5"/>
-      <c r="B39" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F39" s="6" t="s">
+      <c r="D40" s="7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="5"/>
-      <c r="B40" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D40" s="8" t="s">
+      <c r="E40" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="F40" s="6" t="s">
+    </row>
+    <row r="41" spans="1:6" ht="111.6" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="5" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="5"/>
-      <c r="B41" s="6" t="s">
+      <c r="C41" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D41" s="8" t="s">
+      <c r="E41" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="F41" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="F41" s="6" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="5" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="5"/>
-      <c r="B42" s="6" t="s">
+      <c r="C42" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D42" s="8" t="s">
+      <c r="E42" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="F42" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="F42" s="6" t="s">
+    </row>
+    <row r="43" spans="1:6" ht="167.4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="5" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="5"/>
-      <c r="B43" s="6" t="s">
+      <c r="C43" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E43" s="6" t="s">
+      <c r="F43" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="19">
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:A29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:A43"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9 C35 C31:C33 C23 C18 C12" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C12">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C18">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C23">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"replicates_and_mean,mean_only,replicates_only"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"points,line,points+line"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C32">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C35">
-      <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changed settings file to match disabling replicates option
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -201,6 +201,31 @@
     <t>sample_tags</t>
   </si>
   <si>
+    <t>Disabled replicates:</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+List of replicate names. 
+Example: ["1a", "2b", "3c"]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Choose specific replicates to disable from the analysis.
+Disabled replicates are excluded from the analysis by replicate name.
+NOTE #1: each replicate name must be written inside quotes (" ").
+NOTE #2: write replicate names without suffixes.
+Correct example: ["1a", "2b"]
+Incorrect example: ["1a_Raw.csv", "2b_Raw.csv"]
+</t>
+  </si>
+  <si>
+    <t>disabled_replicates</t>
+  </si>
+  <si>
     <t>Include all files:</t>
   </si>
   <si>
@@ -586,9 +611,6 @@
   </si>
   <si>
     <t>Group names:</t>
-  </si>
-  <si>
-    <t>[]</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -657,31 +679,6 @@
   </si>
   <si>
     <t>override_peak_txt_dy</t>
-  </si>
-  <si>
-    <t>Replicates to disable:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Examples:
-• Single replicate:
-[None, None, ["2a"], None]
-• Multiple replicates:
-[None, ["1a", "1b"], ["2c"], None]
-• INCORRECT:
-[None, None, "2a", None]
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-For each group choose specific replicates to disable from the average signal.
-NOTE #1: each value in the outer list has to be either a list or None.
-NOTE #2: each replicate has to be written inside quotes (" ").
-NOTE #3: disabling a replicate also removes it from the plot.
-</t>
-  </si>
-  <si>
-    <t>override_mean_replicate_cols</t>
   </si>
   <si>
     <t>Replicates to hide:</t>
@@ -1289,82 +1286,82 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="20" customHeight="1">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="5" t="s">
+    <row r="10" spans="1:6">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="9">
+      <c r="D10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="20" customHeight="1">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="9">
         <v>25</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="20" customHeight="1">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="E13" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="6" t="s">
+    </row>
+    <row r="14" spans="1:6" ht="20" customHeight="1">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="5"/>
       <c r="B15" s="6" t="s">
         <v>46</v>
       </c>
@@ -1399,116 +1396,116 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="20" customHeight="1">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5" t="s">
+    <row r="17" spans="1:6">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="D17" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="20" customHeight="1">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="5" t="s">
+      <c r="F17" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="6" t="s">
+    </row>
+    <row r="18" spans="1:6" ht="20" customHeight="1">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="9">
+      <c r="B19" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="20" customHeight="1">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="9">
         <v>10</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="7"/>
       <c r="D21" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="20" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="6" t="s">
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E23" s="6" t="s">
+      <c r="C22" s="7"/>
+      <c r="D22" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>72</v>
       </c>
+      <c r="F22" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="20" customHeight="1">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="5"/>
+      <c r="A24" s="5" t="s">
+        <v>74</v>
+      </c>
       <c r="B24" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>76</v>
@@ -1540,214 +1537,214 @@
       <c r="B26" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="7"/>
+      <c r="C26" s="7" t="s">
+        <v>84</v>
+      </c>
       <c r="D26" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="5"/>
       <c r="B27" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="5"/>
       <c r="B28" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" s="9">
-        <v>0</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="C28" s="7"/>
       <c r="D28" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="5"/>
       <c r="B29" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C29" s="9">
         <v>0</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="20" customHeight="1">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B31" s="6" t="s">
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="5"/>
+      <c r="B30" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C31" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E31" s="6" t="s">
+      <c r="C30" s="9">
+        <v>0</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>102</v>
       </c>
+      <c r="F30" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="20" customHeight="1">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="5"/>
+      <c r="A32" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="B32" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="5"/>
       <c r="B33" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="20" customHeight="1">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B35" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" s="6" t="s">
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="5"/>
+      <c r="B34" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="C34" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>112</v>
       </c>
+      <c r="F34" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="20" customHeight="1">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="5"/>
+      <c r="A36" s="5" t="s">
+        <v>114</v>
+      </c>
       <c r="B36" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C36" s="9">
+        <v>115</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="5"/>
+      <c r="B37" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C37" s="9">
         <v>2</v>
       </c>
-      <c r="D36" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="20" customHeight="1">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C38" s="7" t="s">
+      <c r="D37" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="E37" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F38" s="6" t="s">
+    </row>
+    <row r="38" spans="1:6" ht="20" customHeight="1">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="5" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5"/>
       <c r="B39" s="6" t="s">
         <v>123</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>124</v>
@@ -1762,28 +1759,28 @@
     <row r="40" spans="1:6">
       <c r="A40" s="5"/>
       <c r="B40" s="6" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="5"/>
       <c r="B41" s="6" t="s">
-        <v>130</v>
+        <v>92</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>131</v>
@@ -1801,7 +1798,7 @@
         <v>134</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>135</v>
@@ -1819,7 +1816,7 @@
         <v>138</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>139</v>
@@ -1837,44 +1834,41 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:A29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A39:A43"/>
   </mergeCells>
   <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C10">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C13">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C18">
-      <formula1>"True,False"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C23">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C19">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25">
       <formula1>"replicates_and_mean,mean_only,replicates_only"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C25">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C26">
       <formula1>"points,line,points+line"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
-      <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C32">
       <formula1>"True,False"</formula1>
@@ -1882,7 +1876,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C35">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C34">
+      <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C36">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimized settings file interface
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
   <si>
     <t>Section</t>
   </si>
@@ -175,8 +175,8 @@
   <si>
     <t xml:space="preserve">
 How many raw files belong to each sample/group.
-Note that the code assumes the replicates are saved consecutively.
-For example, if each sample has 3 replicate files, use 3.
+They are grouped by their order in your folder.
+For example, if each sample has 4 replicate files, use 4.
 </t>
   </si>
   <si>
@@ -194,7 +194,6 @@
   <si>
     <t xml:space="preserve">
 Optional labels for each group of replicates. These names will be assigned to groups according to the detected file order.
-If no labels are provided, the groups will be named automatically: "Unlabeled_1", "Unlabeled_2", "Unlabeled_3", ...
 </t>
   </si>
   <si>
@@ -215,7 +214,6 @@
   <si>
     <t xml:space="preserve">
 Choose specific replicates to disable from the analysis.
-Disabled replicates are excluded from the analysis by replicate name.
 NOTE #1: each replicate name must be written inside quotes (" ").
 NOTE #2: write replicate names without suffixes.
 Correct example: ["1a", "2b"]
@@ -238,7 +236,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-Handle the extra files that don't complete a full group of replicates: 
+Handle the extra files that don't complete a full group: 
 •  False = ignore leftover files and print a message to the user.
 •  True = analyse leftover files as an additional group named Extra.
 </t>
@@ -427,6 +425,45 @@
     <t>show_average_peaks_txt</t>
   </si>
   <si>
+    <t>GROUP-SPECIFIC OVERRIDES</t>
+  </si>
+  <si>
+    <t>Group names:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+List of group names. 
+Example: ["Liver", "Lung"]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Use this section only when you want to limit Y-axis differently for specific groups.
+For example, if group names are ["Liver", "Lung"], then [500, 700] means:Liver gets 500, and Lung gets 700.
+NOTE: each group name MUST be in quotes (example: "Liver").Each position matches the group name in the same position.
+</t>
+  </si>
+  <si>
+    <t>override_group_names</t>
+  </si>
+  <si>
+    <t>Y-axis limit:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+List with limits (number/range).
+Example: [500, (-100, 500)]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+When choosing a limit, maintain the same order in which you listed the groups.
+</t>
+  </si>
+  <si>
+    <t>override_y_limit</t>
+  </si>
+  <si>
     <t>PEAK/PERIOD TABLE SETTINGS</t>
   </si>
   <si>
@@ -442,23 +479,6 @@
     <t>save_peak_tables</t>
   </si>
   <si>
-    <t>Peak table decimals:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Non-negative integer. 
-Example: 2
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Number of decimals in peak and period values.
-</t>
-  </si>
-  <si>
-    <t>peak_table_decimals</t>
-  </si>
-  <si>
     <t>DATA LENGTH / TAIL CUTTING</t>
   </si>
   <si>
@@ -529,69 +549,6 @@
     <t>remove_noise</t>
   </si>
   <si>
-    <t>FILE SETTINGS</t>
-  </si>
-  <si>
-    <t>File extension:</t>
-  </si>
-  <si>
-    <t>.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-File extension. 
-Example .csv
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Usually this should not be changed. Change only if the Lumi output files use a different file extension.
-</t>
-  </si>
-  <si>
-    <t>extension</t>
-  </si>
-  <si>
-    <t>Suffix to remove:</t>
-  </si>
-  <si>
-    <t>_Raw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Text suffix. 
-Example: _Raw
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Usually this should not be changed. This suffix is removed from raw file names when creating cleaner names.
-</t>
-  </si>
-  <si>
-    <t>suffix_to_remove</t>
-  </si>
-  <si>
-    <t>Raw file suffix:</t>
-  </si>
-  <si>
-    <t>_Raw.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Text suffix. 
-Example: _Raw.csv
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Usually this should not be changed. Change only if the Lumi output files use different names.
-</t>
-  </si>
-  <si>
-    <t>file_suffix</t>
-  </si>
-  <si>
     <t>SAVING</t>
   </si>
   <si>
@@ -605,97 +562,6 @@
   </si>
   <si>
     <t>save_file</t>
-  </si>
-  <si>
-    <t>GROUP-SPECIFIC OVERRIDES</t>
-  </si>
-  <si>
-    <t>Group names:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-List of group names. 
-Example: ["Liver", "Kidney", "Lung"]
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Use this section only when you want to override specific settings for specific groups.
-Important Notes:
-NOTE #1: write only the groups for which you want to override at least one setting.
-NOTE #2: each group name MUST be in quotes (example: "Liver").
-NOTE #3: when overriding a setting, maintain the same order in which you listed the groups.Each position matches the group name in the same position.
-For example, if group names are ["Liver", "Kidney", "Lung"], then [500, None, 700] means:
-Liver gets 500, Kidney gets no override, and Lung gets 700.
-</t>
-  </si>
-  <si>
-    <t>override_group_names</t>
-  </si>
-  <si>
-    <t>Y-axis limit:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-List with one value (number/range) per group, or None for no override.
-Example: [500, None, (-100, 500)]
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-See section: PLOTTING SETTINGS, setting: Y-axis limit, for a detailed description.
-</t>
-  </si>
-  <si>
-    <t>override_y_limit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-List with one value per group, or None for no override. 
-Example: ["Exp. 1", None, None, None]
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-See section: PLOTTING SETTINGS, setting: Plot description, for a detailed description.
-</t>
-  </si>
-  <si>
-    <t>override_description</t>
-  </si>
-  <si>
-    <t>Peak label vertical offset:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-List with one value per group, or None for no override. 
-Example: [20, None, None, 35]
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-This value is used to adjust the position of the peak text labels.
-</t>
-  </si>
-  <si>
-    <t>override_peak_txt_dy</t>
-  </si>
-  <si>
-    <t>Replicates to hide:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-See examples above.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-For each group choose specific replicates to hide from the plot.
-NOTE: this does NOT exclude them from the calculation of the average signal.
-</t>
-  </si>
-  <si>
-    <t>override_visible_replicate_cols</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -1516,34 +1382,34 @@
         <v>78</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="5"/>
       <c r="B25" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C25" s="9">
-        <v>2</v>
+        <v>82</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="20" customHeight="1">
@@ -1556,16 +1422,16 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C27" s="9">
-        <v>10</v>
+        <v>87</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>88</v>
@@ -1574,40 +1440,40 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
+    <row r="28" spans="1:6" ht="20" customHeight="1">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="8" t="s">
+      <c r="B29" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="C29" s="9">
+        <v>10</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="20" customHeight="1">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
+      <c r="F29" s="6" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="5" t="s">
-        <v>94</v>
-      </c>
+      <c r="A30" s="5"/>
       <c r="B30" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="9">
-        <v>25</v>
-      </c>
+      <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
         <v>96</v>
       </c>
@@ -1618,219 +1484,83 @@
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="5"/>
-      <c r="B31" s="6" t="s">
+    <row r="31" spans="1:6" ht="20" customHeight="1">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="B32" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="9">
+        <v>25</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="5"/>
+      <c r="B33" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D33" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="20" customHeight="1">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F33" s="6" t="s">
+    </row>
+    <row r="34" spans="1:6" ht="20" customHeight="1">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="5" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="5"/>
-      <c r="B34" s="6" t="s">
+      <c r="B35" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="F35" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="5"/>
-      <c r="B35" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="20" customHeight="1">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="20" customHeight="1">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="5"/>
-      <c r="B40" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="5"/>
-      <c r="B41" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="5"/>
-      <c r="B42" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="5"/>
-      <c r="B43" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <mergeCells count="19">
+  <mergeCells count="16">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A6:F6"/>
@@ -1842,14 +1572,11 @@
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A39:A43"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A34:F34"/>
   </mergeCells>
   <dataValidations count="10">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C10">
@@ -1873,13 +1600,13 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C22">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C27">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C37">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C35">
       <formula1>"True,False"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimized settings file interface + bugs fixed
</commit_message>
<xml_diff>
--- a/settings.xlsx
+++ b/settings.xlsx
@@ -214,8 +214,7 @@
   <si>
     <t xml:space="preserve">
 Choose specific replicates to disable from the analysis.
-NOTE #1: each replicate name must be written inside quotes (" ").
-NOTE #2: write replicate names without suffixes.
+NOTE: each replicate name must be written inside quotes (" ").
 Correct example: ["1a", "2b"]
 Incorrect example: ["1a_Raw.csv", "2b_Raw.csv"]
 </t>
@@ -425,7 +424,7 @@
     <t>show_average_peaks_txt</t>
   </si>
   <si>
-    <t>GROUP-SPECIFIC OVERRIDES</t>
+    <t>SPECIFIC Y-AXIS LIMITS</t>
   </si>
   <si>
     <t>Group names:</t>
@@ -438,8 +437,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-Use this section only when you want to limit Y-axis differently for specific groups.
-For example, if group names are ["Liver", "Lung"], then [500, 700] means:Liver gets 500, and Lung gets 700.
+Use this section only when you want to limit Y-axis differently for specific groups.For example, if group names are ["Liver", "Lung"], then [500, 700] means:Liver gets 500, and Lung gets 700.
 NOTE: each group name MUST be in quotes (example: "Liver").Each position matches the group name in the same position.
 </t>
   </si>
@@ -464,6 +462,91 @@
     <t>override_y_limit</t>
   </si>
   <si>
+    <t>DATA LENGTH / TAIL CUTTING</t>
+  </si>
+  <si>
+    <t>Length of Lumi's interval:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Positive number. 
+Example: 10
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+The length of the sampling interval in minutes. 
+NOTE: Lumi's interval by default is 10 minutes.
+</t>
+  </si>
+  <si>
+    <t>interval_minutes</t>
+  </si>
+  <si>
+    <t>Maximum days to analyze:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Positive number, or None.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Limit analysis to the first N days. Leave None for no limit, or choose a positive number N for number of days to analyze.
+This feature is useful to cut the tail of the data if it isn't significant to the analysis.
+</t>
+  </si>
+  <si>
+    <t>max_days</t>
+  </si>
+  <si>
+    <t>ANALYSIS SETTINGS</t>
+  </si>
+  <si>
+    <t>Maximum background noise:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Number. 
+Example: 25
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+The minimum counts/sec value that marks the beginning of the real signal.All consecutive rows from the start, with counts below this threshold, are treated as pre-sample noise.
+</t>
+  </si>
+  <si>
+    <t>noise_max</t>
+  </si>
+  <si>
+    <t>Remove background noise:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+•  True = subtract the average pre-sample noise from the signal.
+•  False = keep the signal without subtracting that background.
+</t>
+  </si>
+  <si>
+    <t>remove_noise</t>
+  </si>
+  <si>
+    <t>SAVING</t>
+  </si>
+  <si>
+    <t>Save processed files:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+•  True = save processed files to the given output folder.
+•  False = run analysis without saving files.
+</t>
+  </si>
+  <si>
+    <t>save_file</t>
+  </si>
+  <si>
     <t>PEAK/PERIOD TABLE SETTINGS</t>
   </si>
   <si>
@@ -477,91 +560,6 @@
   </si>
   <si>
     <t>save_peak_tables</t>
-  </si>
-  <si>
-    <t>DATA LENGTH / TAIL CUTTING</t>
-  </si>
-  <si>
-    <t>Length of Lumi's interval:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Positive number. 
-Example: 10
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-The length of the sampling interval in minutes. 
-NOTE: Lumi's interval by default is 10 minutes.
-</t>
-  </si>
-  <si>
-    <t>interval_minutes</t>
-  </si>
-  <si>
-    <t>Maximum days to analyze:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Positive number, or None.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Limit analysis to the first N days. Leave None for no limit, or choose a positive number N for number of days to analyze.
-This feature is useful to cut the tail of the data if it isn't significant to the analysis.
-</t>
-  </si>
-  <si>
-    <t>max_days</t>
-  </si>
-  <si>
-    <t>ANALYSIS SETTINGS</t>
-  </si>
-  <si>
-    <t>Maximum background noise:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Number. 
-Example: 25
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-The minimum counts/sec value that marks the beginning of the real signal.All consecutive rows from the start, with counts below this threshold, are treated as pre-sample noise.
-</t>
-  </si>
-  <si>
-    <t>noise_max</t>
-  </si>
-  <si>
-    <t>Remove background noise:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-•  True = subtract the average pre-sample noise from the signal.
-•  False = keep the signal without subtracting that background.
-</t>
-  </si>
-  <si>
-    <t>remove_noise</t>
-  </si>
-  <si>
-    <t>SAVING</t>
-  </si>
-  <si>
-    <t>Save processed files:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-•  True = save processed files to the given output folder.
-•  False = run analysis without saving files.
-</t>
-  </si>
-  <si>
-    <t>save_file</t>
   </si>
 </sst>
 </file>
@@ -1427,93 +1425,93 @@
       <c r="B27" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="9">
+        <v>10</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="20" customHeight="1">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="9">
+        <v>25</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="5"/>
+      <c r="B31" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D31" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="20" customHeight="1">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C29" s="9">
-        <v>10</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="5"/>
-      <c r="B30" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="20" customHeight="1">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C32" s="9">
-        <v>25</v>
-      </c>
-      <c r="D32" s="8" t="s">
+      <c r="E31" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="F32" s="6" t="s">
+    </row>
+    <row r="32" spans="1:6" ht="20" customHeight="1">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="5" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="5"/>
       <c r="B33" s="6" t="s">
         <v>104</v>
       </c>
@@ -1572,10 +1570,10 @@
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:F32"/>
     <mergeCell ref="A34:F34"/>
   </mergeCells>
   <dataValidations count="10">
@@ -1600,7 +1598,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C22">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C27">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C31">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Please choose one of the allowed values." promptTitle="Choose a value" prompt="Choose one of the allowed values." sqref="C33">

</xml_diff>